<commit_message>
ADI-01: ubicación real por fuente + fecha (prom. de archivos); columna 'Fecha de la fuente'
- ubicacion_ruta de las 27 fuentes apuntando a su archivo/carpeta real (incl. F-09/F-18
  imágenes/mínima info); F-23/24/25 a su evidencia externa (Resultados Volumetría,
  Estructura DDL, DataStage). Ninguna fuente sin evidencia → no se descarta ninguna.
- fecha_version_estado = fecha promedio de los archivos de la fuente; se dropea
  versión/estado (no poblables). Grid y generador relabelados a 'Fecha de la fuente'.
- Excel de descarga regenerados en vivo (incl. ADI-01) + zip.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-01.xlsx
+++ b/client/public/artefactos/ADI-01.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Fecha / versión / estado</t>
+          <t>Fecha de la fuente</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\D-01 - Terminos de Referencia del servicio.pdf</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-01 - Terminos de Referencia del servicio.pdf</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\D-02 - Plan de Trabajo del DE de la BDI.docx</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-02 - Plan de Trabajo del DE de la BDI.docx</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\D-03 - Mapa de Procesos ONP 2026.pdf</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-03 - Mapa de Procesos ONP 2026.pdf</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\D-04 - Cadena de Valor ONP 2026.pdf</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-04 - Cadena de Valor ONP 2026.pdf</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\D-06 - Inventarios preliminares (BD, Servidores, APP)\</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-05 - Inventarios preliminares (BD, Servidores, APP)</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\D-07 - Documentos de Arquitectura de Aplicaciones\</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-06 - Documentos de Arquitectura de Aplicaciones</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-01 - Matriz de Interesados de la ONP.xlsx</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-07 - Matriz de Interesados de la ONP.xlsx</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-03 - Formatos oficiales de artefactos (Plantillas_Artefactos_ONP).xlsx</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-08 - Formatos oficiales de artefactos (Plantillas_Artefactos_ONP).xlsx</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Pendiente de entrega · P1</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Pendiente de entrega</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-09 - Arquitectura Referencial Institucional</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Parcialmente disponible · P1</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-05 - Procesos (diagramas e inventario parcial)\</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-10 - Procesos (diagramas e inventario parcial)</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Parcialmente disponible · P1</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-07 - Modelos de Datos (parcial)\</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-11 - Modelos de Datos (parcial)</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Parcialmente disponible · P1</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-10 - Seguridad de la informacion (politicas y directivas)\</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-12 - Seguridad de la informacion (politicas y directivas)</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-11 - Inventario de servidores de BD.xlsx</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-13 - Inventario de servidores de BD.xlsx</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-10-05 / vigente</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-14 - Inventario de BD_20261005.xlsx</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-14 - Inventario de BD_20261005.xlsx</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-13 - Inventario de APP.xlsx</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-15 - Inventario de APP.xlsx</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-14 - Inventario de DB Links\</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-16 - Inventario de DB Links</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-15 - ETL, jobs, mallas y tareas programadas\</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-17 - ETL, jobs, mallas y tareas programadas</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Pendiente de entrega · P1</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Pendiente de entrega</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-18 - Interoperabilidad (PIDE y externas)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-18 - Estudio de preinversion - ONPDigital ProyectoInversion.pdf</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-19 - Estudio de preinversion - ONPDigital ProyectoInversion.pdf</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-20 - Cronograma ONP v0.2.xlsx</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-20 - Cronograma ONP v0.2.xlsx</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Parcialmente disponible · P2</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\F-27 - Licenciamiento Oracle (parcial)\</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-21 - Licenciamiento Oracle (parcial)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Disponible · P1</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Fuentes (Google Drive)</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-22 - Reuniones de levantamiento</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-10-27 · Disponible</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-10-27 · Disponible</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Estructura DDL\\</t>
+          <t>Estructura DDL</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-10-27 · Disponible</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>DataStage\\ ; ARQUITECTURA OTI...\\DBLINKS</t>
+          <t>DataStage</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-18 · Disponible (proyecto)</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01\\F-26 - Modelo Conceptual del SIIP</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-23 - Modelo Conceptual del SIIP</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-10-28 / vigente</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Fuentes de Informacion ADI-01/F-27 - Volumetria y metadata Oracle (extraccion DBA en vivo)/</t>
+          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-27 - Volumetria y metadata Oracle (extraccion DBA en vivo)</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">

</xml_diff>

<commit_message>
ADI-01: carpetas F-24/F-25 con evidencia, Evidencia=archivo/patrón para todas, quita col Ubicación
- Creadas carpetas de fuente para F-24 (Estructura física: 26 instancias .txt + 19G8/PR2 .csv)
  y F-25 (DataStage: .dsx + xlsx + csv) en la carpeta de fuentes (para subir a Drive)
- evidencia_revision = nombre de archivo o patrón/glob (por extensión+prefijo) para las 27
- Columna "Ubicación / ruta" retirada del artefacto (la ubicación la da el enlace a la nube)
- Excel de descarga regenerado en vivo (ADI-01 = 15 cols) + zip

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-01.xlsx
+++ b/client/public/artefactos/ADI-01.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,20 +486,15 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Ubicación / ruta</t>
+          <t>Evidencia (archivo/patrón)</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Evidencia</t>
+          <t>Enlace</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
-        <is>
-          <t>Enlace</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
         <is>
           <t>Origen</t>
         </is>
@@ -568,20 +563,15 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-01 - Terminos de Referencia del servicio.pdf</t>
+          <t>F-01 - Terminos de Referencia del servicio.pdf</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Documento TDR del servicio</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -650,20 +640,15 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-02 - Plan de Trabajo del DE de la BDI.docx</t>
+          <t>F-02 - Plan de Trabajo del DE de la BDI.docx</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Plan de Trabajo (Primer Entregable)</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -732,20 +717,15 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-03 - Mapa de Procesos ONP 2026.pdf</t>
+          <t>F-03 - Mapa de Procesos ONP 2026.pdf</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Mapa de Procesos ONP 2026</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -814,20 +794,15 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-04 - Cadena de Valor ONP 2026.pdf</t>
+          <t>F-04 - Cadena de Valor ONP 2026.pdf</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Cadena de Valor ONP 2026</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -896,20 +871,15 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-05 - Inventarios preliminares (BD, Servidores, APP)</t>
+          <t>*.xlsx (5)</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Inventarios 01/02/03</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -978,20 +948,15 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-06 - Documentos de Arquitectura de Aplicaciones</t>
+          <t>Documento de Arquitectura*.pdf (16)</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Documentos de arquitectura (D-07)</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1060,20 +1025,15 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-07 - Matriz de Interesados de la ONP.xlsx</t>
+          <t>F-07 - Matriz de Interesados de la ONP.xlsx</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Solicitud a UE 003 · revisor: Jefe de Proyecto</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1142,20 +1102,15 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-08 - Formatos oficiales de artefactos (Plantillas_Artefactos_ONP).xlsx</t>
+          <t>F-08 - Formatos oficiales de artefactos (Plantillas_Artefactos_ONP).xlsx</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Solicitud a UE 003 · revisor: Jefe de Proyecto</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1224,20 +1179,15 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-09 - Arquitectura Referencial Institucional</t>
+          <t>*.pptx (3) · *.jpg (2)</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: Arq. Datos / Consultor Sr. TI</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1306,20 +1256,15 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-10 - Procesos (diagramas e inventario parcial)</t>
+          <t>Aplicaciones - Procesos de tipo soporte.xlsx · Diagrama_General_Procesos.drawio</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Solicitud a OPPM · revisor: Arq. Datos / Consultor Funcional</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1388,20 +1333,15 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-11 - Modelos de Datos (parcial)</t>
+          <t>*.doc (141) · *.zip (11) · *.docx (10) · diagrama.erx*.erx (2) · *.pdf (2) · CAPACITACION*.pptx (2) · Catalogo de Aplicaciones OTI.DE.xlsx</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: Arq. Datos / DBA Senior</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1470,20 +1410,15 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-12 - Seguridad de la informacion (politicas y directivas)</t>
+          <t>*.pdf (7)</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: Arq. de Datos</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1552,20 +1487,15 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-13 - Inventario de servidores de BD.xlsx</t>
+          <t>F-13 - Inventario de servidores de BD.xlsx</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: DBA Senior</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1634,20 +1564,15 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-14 - Inventario de BD_20261005.xlsx</t>
+          <t>F-14 - Inventario de BD_20261005.xlsx</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Archivo 02__Inventario_de_BD_20261005.xlsx (OTI) · revisor DBA Senior</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1716,20 +1641,15 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-15 - Inventario de APP.xlsx</t>
+          <t>F-15 - Inventario de APP.xlsx</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: DBA Senior / Arq. Datos</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1798,20 +1718,15 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-16 - Inventario de DB Links</t>
+          <t>*.vsd (7) · dblinks*.xlsx (4)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: DBA Senior</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1880,20 +1795,15 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-17 - ETL, jobs, mallas y tareas programadas</t>
+          <t>crontab*.txt (72) · Reporte*.xls (8) · *.xlsx (6)</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: DBA Senior</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -1962,20 +1872,15 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-18 - Interoperabilidad (PIDE y externas)</t>
+          <t>Modelo de datos.docx</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: DBA Senior / Arq. Datos</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -2044,20 +1949,15 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-19 - Estudio de preinversion - ONPDigital ProyectoInversion.pdf</t>
+          <t>F-19 - Estudio de preinversion - ONPDigital ProyectoInversion.pdf</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Solicitud a UE 003 · revisor: Esp. Doc. Equivalente</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -2126,20 +2026,15 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-20 - Cronograma ONP v0.2.xlsx</t>
+          <t>F-20 - Cronograma ONP v0.2.xlsx</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Solicitud a UE 003 · revisor: Esp. Doc. Equivalente</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -2208,20 +2103,15 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-21 - Licenciamiento Oracle (parcial)</t>
+          <t>Oracle - Product*.png (2) · Ayuda_memoria_analisis_licenciamiento_Oracle_ONP.docx · Uso de licencias.xlsx</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Solicitud a OTI · revisor: Consultor Sr. TI</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -2290,20 +2180,15 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-22 - Reuniones de levantamiento</t>
+          <t>[ONP-DE_BDI] Reunión de Levantamiento de Información (*.docx (7)</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>7 actas de reunión</t>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
         <is>
           <t>ADI-01</t>
         </is>
@@ -2372,16 +2257,11 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Resultados de scripts de Volumetria</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>SQLSERVER_V2.xlsx; VOLUMETRIA_ORACLE/MYSQL/DB2</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr">
+          <t>*.txt (47) · SQLSERVER*.xlsx (2) · VOLUMETRIA_DB2.rar · VOLUMETRIA_SQLSERVER.docx</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
         <is>
           <t>nueva (LCP)</t>
         </is>
@@ -2415,7 +2295,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2450,16 +2330,11 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Estructura DDL</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>&lt;BD&gt;_&lt;ts&gt;.txt/.csv por instancia</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
+          <t>*.txt (25) · *.csv (2)</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
         <is>
           <t>nueva (LCP)</t>
         </is>
@@ -2493,7 +2368,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2528,16 +2403,11 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>DataStage</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>FUENTES_EXTERNAS/INTERNAS/PARAMETROS.dsx; dblinks_produccion_ordenado.xlsx</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr">
+          <t>*.dsx (3) · *.xlsx (2) · integraciones_datastage_raw.csv</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
         <is>
           <t>nueva (LCP)</t>
         </is>
@@ -2606,16 +2476,11 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-23 - Modelo Conceptual del SIIP</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>MC SIIP 20260918...PROYECTO.docx</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr">
+          <t>MC SIIP 20260918SDP  M-102-DPD.SPD_PROYECTO.docx</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
         <is>
           <t>nueva (LCP)</t>
         </is>
@@ -2684,16 +2549,11 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Propuestas E2 - LCP\Fuentes de Informacion ADI-01\F-27 - Volumetria y metadata Oracle (extraccion DBA en vivo)</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Script extrae_metadata_oracle.py + load_metadata_oracle.py (repo Modelo_BDI)</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr">
+          <t>*.xlsx (11) · *.zip (2)</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr">
         <is>
           <t>nueva (LCP)</t>
         </is>

</xml_diff>

<commit_message>
ADI-01: enlace Drive común para las 27, quita columna Origen, F-26/F-23 como carpetas visibles
- Todas las fuentes con el mismo enlace a la carpeta Drive
- Columna "Origen" retirada del artefacto
- SIIP renombrado a 'F-26 - Modelo Conceptual del SIIP'; creada 'F-23 - Volumetria
  ejecutada por ONP' → F-01..F-27 todas como carpeta/archivo visibles para subir a Drive
- Excel de descarga regenerado (ADI-01 = 14 cols)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-01.xlsx
+++ b/client/public/artefactos/ADI-01.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,11 +494,6 @@
           <t>Enlace</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Origen</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -571,11 +566,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -648,11 +638,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -725,11 +710,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -802,11 +782,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -879,11 +854,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -956,11 +926,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1033,11 +998,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1110,11 +1070,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1187,11 +1142,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1264,11 +1214,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1341,11 +1286,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1418,11 +1358,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1495,11 +1430,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1572,11 +1502,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1649,11 +1574,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1726,11 +1646,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1803,11 +1718,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1880,11 +1790,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1957,11 +1862,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2034,11 +1934,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2111,11 +2006,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2188,11 +2078,6 @@
           <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>ADI-01</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2222,7 +2107,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2260,10 +2145,9 @@
           <t>*.txt (47) · SQLSERVER*.xlsx (2) · VOLUMETRIA_DB2.rar · VOLUMETRIA_SQLSERVER.docx</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>nueva (LCP)</t>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
     </row>
@@ -2333,10 +2217,9 @@
           <t>*.txt (25) · *.csv (2)</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>nueva (LCP)</t>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
     </row>
@@ -2406,10 +2289,9 @@
           <t>*.dsx (3) · *.xlsx (2) · integraciones_datastage_raw.csv</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>nueva (LCP)</t>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
     </row>
@@ -2479,10 +2361,9 @@
           <t>MC SIIP 20260918SDP  M-102-DPD.SPD_PROYECTO.docx</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>nueva (LCP)</t>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
     </row>
@@ -2552,10 +2433,9 @@
           <t>*.xlsx (11) · *.zip (2)</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>nueva (LCP)</t>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1-_tyMB6DMqmpdQZf62m6pcuJwUfwCDAq</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ADI-04: Vacíos/solapamientos/dispersión y Observaciones modelo conceptual como texto analítico (0 columnas manuales); F-08 corregida
- dominio_funcional.obs_vacios / obs_modelo_concept: narrativa por dominio (cobertura/vacíos/
  solapamiento/dispersión y entidad que aporta + candidata a maestro), marcada *; analisis_dominio_adi04.py
- col 13 renombrada a nombre oficial TDR "Vacíos / solapamientos / dispersión"
- F-08 reetiquetada: no son formatos oficiales ONP sino plantillas LCP con el mínimo requerido en los TDR

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-01.xlsx
+++ b/client/public/artefactos/ADI-01.xlsx
@@ -1007,7 +1007,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Formatos oficiales de artefactos ADI, AMC y ADE</t>
+          <t>Formatos de artefactos ADI/AMC/ADE (plantillas LCP con el mínimo del TDR)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1017,12 +1017,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Plantillas oficiales ONP de los artefactos ADI/AMC/ADE; definen la estructura y columnas esperadas de cada entregable.</t>
+          <t>Plantillas de los artefactos generadas por LCP a partir de la información mínima requerida en los TDR (no son formatos oficiales de ONP); definen la estructura/columnas esperadas de cada entregable.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>UE 003</t>
+          <t>LCP (Firma Consultora)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Metodológica (plantillas)</t>
+          <t>Metodológica (plantillas LCP)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Define las COLUMNAS de cada artefacto (aporte total al diseño de ADI-01..09) y es la base del mapeo de trazabilidad columna↔fuente.</t>
+          <t>Define las columnas mínimas (según TDR) de cada artefacto ADI-01..09; base del mapeo de trazabilidad columna↔fuente.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">

</xml_diff>